<commit_message>
bush medicine, bush tucker websites and updated person metadata
</commit_message>
<xml_diff>
--- a/test_data/gurindji_yawu/data/metadata_new.xlsx
+++ b/test_data/gurindji_yawu/data/metadata_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abby/Documents/Work/PosterWebsites/ro-crate-html-lite/test_data/gurindji_yawu/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B40FF50D-297F-1F4A-BF9B-9DBC72783F1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E6B574-F217-6F48-A0BD-768BC4C6E93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="253">
   <si>
     <t>name</t>
   </si>
@@ -819,9 +819,6 @@
   </si>
   <si>
     <t>Person</t>
-  </si>
-  <si>
-    <t>isRef_person</t>
   </si>
   <si>
     <t>about/speaker-headshots/VioletWadrill.jpg</t>
@@ -2856,7 +2853,7 @@
     </row>
     <row r="53" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B53" t="s">
         <v>27</v>
@@ -2867,7 +2864,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
@@ -2878,7 +2875,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B55" t="s">
         <v>27</v>
@@ -2889,7 +2886,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B56" t="s">
         <v>27</v>
@@ -3110,7 +3107,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
@@ -3118,7 +3115,7 @@
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -3131,14 +3128,11 @@
       <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -3152,13 +3146,10 @@
         <v>248</v>
       </c>
       <c r="E2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>172</v>
       </c>
@@ -3172,13 +3163,10 @@
         <v>248</v>
       </c>
       <c r="E3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="13" x14ac:dyDescent="0.2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>181</v>
       </c>
@@ -3192,13 +3180,10 @@
         <v>248</v>
       </c>
       <c r="E4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>199</v>
       </c>
@@ -3212,10 +3197,7 @@
         <v>248</v>
       </c>
       <c r="E5" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
lower res images and new audio
</commit_message>
<xml_diff>
--- a/test_data/gurindji_yawu/data/metadata_new.xlsx
+++ b/test_data/gurindji_yawu/data/metadata_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abby/Documents/Work/PosterWebsites/ro-crate-html-lite/test_data/gurindji_yawu/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E6B574-F217-6F48-A0BD-768BC4C6E93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97DBB81F-3D63-3A4E-80C4-A972699AC311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17280" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="1" r:id="rId1"/>
@@ -683,9 +683,6 @@
     <t>files/audio/names/yamanangmanang_BW.mp3</t>
   </si>
   <si>
-    <t>files/audio/names/karralpirnang_VW.mp3.mp3</t>
-  </si>
-  <si>
     <t>files/audio/names/kinyang_VW.mp3</t>
   </si>
   <si>
@@ -831,6 +828,9 @@
   </si>
   <si>
     <t>about/speaker-headshots/TopsyDodd.jpg</t>
+  </si>
+  <si>
+    <t>files/audio/names/karralpirnang_VW.mp3</t>
   </si>
 </sst>
 </file>
@@ -1297,7 +1297,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1305,7 +1305,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -1393,7 +1393,7 @@
         <v>13</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>14</v>
@@ -1411,7 +1411,7 @@
         <v>18</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>19</v>
@@ -1426,7 +1426,7 @@
         <v>22</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="160" x14ac:dyDescent="0.2">
@@ -1474,7 +1474,7 @@
         <v>188</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="224" x14ac:dyDescent="0.2">
@@ -1954,7 +1954,7 @@
         <v>124</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="O12" s="3" t="s">
         <v>178</v>
@@ -1963,7 +1963,7 @@
         <v>178</v>
       </c>
       <c r="Q12" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="128" x14ac:dyDescent="0.2">
@@ -2008,7 +2008,7 @@
         <v>133</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>203</v>
+        <v>252</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>170</v>
@@ -2056,7 +2056,7 @@
         <v>134</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P14" s="3" t="s">
         <v>176</v>
@@ -2089,7 +2089,7 @@
         <v>25</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>141</v>
@@ -2107,7 +2107,7 @@
         <v>166</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>169</v>
@@ -2152,10 +2152,10 @@
         <v>148</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P16" s="3" t="s">
         <v>185</v>
@@ -2197,16 +2197,16 @@
         <v>153</v>
       </c>
       <c r="L17" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="M17" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="M17" s="3" t="s">
-        <v>211</v>
-      </c>
       <c r="N17" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>187</v>
@@ -2251,10 +2251,10 @@
         <v>164</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="P18" s="3" t="s">
         <v>168</v>
@@ -2298,7 +2298,7 @@
         <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2309,7 +2309,7 @@
         <v>27</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2320,7 +2320,7 @@
         <v>27</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2331,7 +2331,7 @@
         <v>27</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2342,7 +2342,7 @@
         <v>27</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2353,7 +2353,7 @@
         <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2364,7 +2364,7 @@
         <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2375,7 +2375,7 @@
         <v>27</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2386,7 +2386,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2397,7 +2397,7 @@
         <v>27</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2408,7 +2408,7 @@
         <v>27</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2419,7 +2419,7 @@
         <v>27</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2430,7 +2430,7 @@
         <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2441,7 +2441,7 @@
         <v>27</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
@@ -2452,7 +2452,7 @@
         <v>27</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2463,7 +2463,7 @@
         <v>27</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2474,7 +2474,7 @@
         <v>27</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2485,7 +2485,7 @@
         <v>27</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2496,7 +2496,7 @@
         <v>27</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2507,7 +2507,7 @@
         <v>27</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2518,7 +2518,7 @@
         <v>27</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2529,7 +2529,7 @@
         <v>27</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2540,7 +2540,7 @@
         <v>27</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2551,7 +2551,7 @@
         <v>27</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2562,7 +2562,7 @@
         <v>27</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2573,7 +2573,7 @@
         <v>27</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2584,7 +2584,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2595,7 +2595,7 @@
         <v>27</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2606,7 +2606,7 @@
         <v>27</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2617,18 +2617,18 @@
         <v>27</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B32" t="s">
         <v>27</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2639,7 +2639,7 @@
         <v>27</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2650,7 +2650,7 @@
         <v>27</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2661,18 +2661,18 @@
         <v>27</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>203</v>
+        <v>252</v>
       </c>
       <c r="B36" t="s">
         <v>27</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2683,7 +2683,7 @@
         <v>27</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2694,18 +2694,18 @@
         <v>27</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B39" t="s">
         <v>27</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2716,7 +2716,7 @@
         <v>27</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2727,18 +2727,18 @@
         <v>27</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B42" t="s">
         <v>27</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2749,29 +2749,29 @@
         <v>27</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B44" t="s">
         <v>27</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B45" t="s">
         <v>27</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2782,29 +2782,29 @@
         <v>27</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B47" t="s">
         <v>27</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B48" t="s">
         <v>27</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2815,29 +2815,29 @@
         <v>27</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B50" t="s">
         <v>27</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B51" t="s">
         <v>27</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16" x14ac:dyDescent="0.2">
@@ -2848,12 +2848,12 @@
         <v>27</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B53" t="s">
         <v>27</v>
@@ -2864,7 +2864,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B54" t="s">
         <v>27</v>
@@ -2875,7 +2875,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B55" t="s">
         <v>27</v>
@@ -2886,7 +2886,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B56" t="s">
         <v>27</v>
@@ -3143,10 +3143,10 @@
         <v>175</v>
       </c>
       <c r="D2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E2" t="s">
         <v>248</v>
-      </c>
-      <c r="E2" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -3160,10 +3160,10 @@
         <v>174</v>
       </c>
       <c r="D3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -3177,10 +3177,10 @@
         <v>183</v>
       </c>
       <c r="D4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
@@ -3194,10 +3194,10 @@
         <v>201</v>
       </c>
       <c r="D5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -3344,7 +3344,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B10" t="s">
         <v>29</v>
@@ -3353,35 +3353,35 @@
         <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>29</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>236</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>29</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>246</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>